<commit_message>
stabalized the script in Create DS & Create Map
</commit_message>
<xml_diff>
--- a/Test Data/Regression/4689052/UK_InHeader_ImportTb.xlsx
+++ b/Test Data/Regression/4689052/UK_InHeader_ImportTb.xlsx
@@ -23,13 +23,13 @@
     <t>Description</t>
   </si>
   <si>
-    <t>2222243_PWE01_1777710138897</t>
-  </si>
-  <si>
-    <t>2222243_PWE02_1777710138897</t>
-  </si>
-  <si>
-    <t>2222243_PWE03_1777710138897</t>
+    <t>2222243_PWE01_1777802282650</t>
+  </si>
+  <si>
+    <t>2222243_PWE02_1777802282650</t>
+  </si>
+  <si>
+    <t>2222243_PWE03_1777802282650</t>
   </si>
   <si>
     <t>Sale of goods, UK</t>

</xml_diff>

<commit_message>
stabalized the Dataset craetion
</commit_message>
<xml_diff>
--- a/Test Data/Regression/4689052/UK_InHeader_ImportTb.xlsx
+++ b/Test Data/Regression/4689052/UK_InHeader_ImportTb.xlsx
@@ -23,13 +23,13 @@
     <t>Description</t>
   </si>
   <si>
-    <t>2222243_PWE01_1777802282650</t>
-  </si>
-  <si>
-    <t>2222243_PWE02_1777802282650</t>
-  </si>
-  <si>
-    <t>2222243_PWE03_1777802282650</t>
+    <t>2222243_PWE01_1777804357663</t>
+  </si>
+  <si>
+    <t>2222243_PWE02_1777804357663</t>
+  </si>
+  <si>
+    <t>2222243_PWE03_1777804357663</t>
   </si>
   <si>
     <t>Sale of goods, UK</t>

</xml_diff>

<commit_message>
Drill functioanlity is added with some Improvements in Dataset creation
</commit_message>
<xml_diff>
--- a/Test Data/Regression/4689052/UK_InHeader_ImportTb.xlsx
+++ b/Test Data/Regression/4689052/UK_InHeader_ImportTb.xlsx
@@ -23,13 +23,13 @@
     <t>Description</t>
   </si>
   <si>
-    <t>2222244_PWE01_1777825842053</t>
-  </si>
-  <si>
-    <t>2222244_PWE02_1777825842053</t>
-  </si>
-  <si>
-    <t>2222244_PWE03_1777825842053</t>
+    <t>2222244_PWE01_1778319778640</t>
+  </si>
+  <si>
+    <t>2222244_PWE02_1778319778640</t>
+  </si>
+  <si>
+    <t>2222244_PWE03_1778319778640</t>
   </si>
   <si>
     <t>Sale of goods, UK</t>

</xml_diff>

<commit_message>
Copying the same script and want to verify in jenkins how much time it will take to execute 5 test
</commit_message>
<xml_diff>
--- a/Test Data/Regression/4689052/UK_InHeader_ImportTb.xlsx
+++ b/Test Data/Regression/4689052/UK_InHeader_ImportTb.xlsx
@@ -23,13 +23,13 @@
     <t>Description</t>
   </si>
   <si>
-    <t>2222244_PWE01_1778319778640</t>
-  </si>
-  <si>
-    <t>2222244_PWE02_1778319778640</t>
-  </si>
-  <si>
-    <t>2222244_PWE03_1778319778640</t>
+    <t>2222244_PWE01_1778649278785</t>
+  </si>
+  <si>
+    <t>2222244_PWE02_1778649278785</t>
+  </si>
+  <si>
+    <t>2222244_PWE03_1778649278785</t>
   </si>
   <si>
     <t>Sale of goods, UK</t>

</xml_diff>